<commit_message>
Schedule delayed actions from runbooks
</commit_message>
<xml_diff>
--- a/data/runbooks/runbook_template.xlsx
+++ b/data/runbooks/runbook_template.xlsx
@@ -365,17 +365,17 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="5">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>host</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>host_group</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.88" customWidth="1" style="6" min="1" max="1"/>
@@ -471,44 +471,49 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="5">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>scope_type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>scope_value</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>trigger_group</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>jira_project</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>jira_issue_type</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>jira_request_type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>delay_minutes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add manual approval for on-call actions
</commit_message>
<xml_diff>
--- a/data/runbooks/runbook_template.xlsx
+++ b/data/runbooks/runbook_template.xlsx
@@ -12,6 +12,7 @@
     <sheet name="actions" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="contacts" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="suppressions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="holidays" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -461,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.88" customWidth="1" style="6" min="1" max="1"/>
@@ -511,9 +512,24 @@
           <t>jira_request_type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>delay_minutes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>approval_when</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>pre_actions</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pre_target</t>
         </is>
       </c>
     </row>
@@ -641,4 +657,70 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="5" min="1" max="1"/>
+    <col width="24" customWidth="1" style="5" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Feriado X</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Independencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Navidad</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>